<commit_message>
FieldCount was returning wrong count. Replaced by RowFieldCount.
</commit_message>
<xml_diff>
--- a/source/Autossential.Workbook.Tests/Samples/OXML_data.xlsx
+++ b/source/Autossential.Workbook.Tests/Samples/OXML_data.xlsx
@@ -4,7 +4,7 @@
   <x:fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <x:workbookPr/>
   <x:bookViews>
-    <x:workbookView windowWidth="28800" windowHeight="12300" tabRatio="500" activeTab="9"/>
+    <x:workbookView windowWidth="28800" windowHeight="12300" activeTab="10"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Header" sheetId="1" r:id="rId1"/>
@@ -17,6 +17,7 @@
     <x:sheet name="Tables" sheetId="8" r:id="rId8"/>
     <x:sheet name="HeadersOnly" sheetId="9" r:id="rId9"/>
     <x:sheet name="EmptyColData" sheetId="10" r:id="rId10"/>
+    <x:sheet name="EmptySheet" sheetId="11" r:id="rId11"/>
   </x:sheets>
   <x:calcPr calcId="191029"/>
   <x:extLst>
@@ -104,9 +105,8 @@
     <r>
       <rPr>
         <sz val="48"/>
-        <color rgb="FF000000"/>
         <rFont val="Avenir Next LT Pro"/>
-        <charset val="1"/>
+        <charset val="134"/>
       </rPr>
       <t>TO-DO</t>
     </r>
@@ -114,18 +114,16 @@
       <rPr>
         <b/>
         <sz val="48"/>
-        <color rgb="FF000000"/>
         <rFont val="Avenir Next LT Pro"/>
-        <charset val="1"/>
+        <charset val="134"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
         <sz val="48"/>
-        <color rgb="FF000000"/>
         <rFont val="Avenir Next LT Pro"/>
-        <charset val="1"/>
+        <charset val="134"/>
       </rPr>
       <t>LIST</t>
     </r>
@@ -323,47 +321,43 @@
   <fonts count="29">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="22"/>
-      <color rgb="FF003366"/>
+      <color indexed="56"/>
       <name val="Avenir Next LT Pro"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="48"/>
-      <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF6600"/>
+      <color indexed="53"/>
       <name val="Avenir Next LT Pro"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color indexed="65"/>
       <name val="Avenir Next LT Pro"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -373,17 +367,17 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color indexed="4"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color indexed="20"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -395,9 +389,9 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color indexed="2"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -413,7 +407,7 @@
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -444,7 +438,7 @@
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -452,7 +446,7 @@
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -460,22 +454,22 @@
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color indexed="65"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -483,50 +477,49 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="48"/>
-      <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="36">
@@ -539,30 +532,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF5CE"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="65"/>
         <bgColor rgb="FFFFF5CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF003366"/>
-        <bgColor rgb="FF333399"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor indexed="56"/>
+        <bgColor indexed="62"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="26"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="47"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -865,171 +858,168 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="178" fontId="7" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="179" fontId="7" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="178" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="7" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -1044,13 +1034,10 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="16" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1138,9 +1125,12 @@
         <color theme="1"/>
       </font>
       <border>
+        <left/>
+        <right/>
         <top style="double">
           <color theme="4"/>
         </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -1185,6 +1175,9 @@
         </patternFill>
       </fill>
       <border>
+        <left/>
+        <right/>
+        <top/>
         <bottom style="thin">
           <color theme="4" tint="0.399975585192419"/>
         </bottom>
@@ -1201,6 +1194,9 @@
         </patternFill>
       </fill>
       <border>
+        <left/>
+        <right/>
+        <top/>
         <bottom style="thin">
           <color theme="4" tint="0.399975585192419"/>
         </bottom>
@@ -1216,6 +1212,9 @@
         <color theme="1"/>
       </font>
       <border>
+        <left/>
+        <right/>
+        <top/>
         <bottom style="thin">
           <color theme="4" tint="0.399975585192419"/>
         </bottom>
@@ -1233,6 +1232,8 @@
         <color theme="1"/>
       </font>
       <border>
+        <left/>
+        <right/>
         <top style="thin">
           <color theme="4"/>
         </top>
@@ -1269,6 +1270,8 @@
         </patternFill>
       </fill>
       <border>
+        <left/>
+        <right/>
         <top style="thin">
           <color theme="4" tint="0.399975585192419"/>
         </top>
@@ -1289,14 +1292,17 @@
         </patternFill>
       </fill>
       <border>
+        <left/>
+        <right/>
+        <top/>
         <bottom style="thin">
           <color theme="4" tint="0.399975585192419"/>
         </bottom>
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+  <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{CA3B9742-4CDE-44DB-9573-93BC8E86ABF0}">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -1305,7 +1311,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{988474DF-EB73-4CCE-8309-EA9124B4F549}">
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="totalRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
@@ -1318,87 +1324,12 @@
       <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFF5CE"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1550,7 +1481,7 @@
       <c r="C2" s="1">
         <v>81847.8</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>44996.6670148727</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -1571,7 +1502,7 @@
       <c r="C3" s="1">
         <v>52317.9</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>45182.6670148843</v>
       </c>
       <c r="E3" s="1" t="s">
@@ -1592,14 +1523,14 @@
       <c r="C4" s="1">
         <v>85773.6</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>45068.6670148843</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" ref="F4:F5" si="0">TRUE()</f>
         <v>1</v>
       </c>
     </row>
@@ -1613,14 +1544,14 @@
       <c r="C5" s="1">
         <v>87183</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>45349.6670148843</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
@@ -1634,7 +1565,7 @@
       <c r="C6" s="1">
         <v>30107.7</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>45054.6670148843</v>
       </c>
       <c r="E6" s="1" t="s">
@@ -1655,7 +1586,7 @@
       <c r="C7" s="1">
         <v>-1908.9</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>45167.6670148843</v>
       </c>
       <c r="E7" s="1" t="s">
@@ -1676,14 +1607,14 @@
       <c r="C8" s="1">
         <v>41974.2</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>44676.6670148843</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" ref="F8:F9" si="1">FALSE()</f>
         <v>0</v>
       </c>
     </row>
@@ -1697,14 +1628,14 @@
       <c r="C9" s="1">
         <v>128266.2</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>45743.6670148843</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1718,14 +1649,14 @@
       <c r="C10" s="1">
         <v>133728.3</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>45378.6670148843</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F10" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" ref="F10:F11" si="2">TRUE()</f>
         <v>1</v>
       </c>
     </row>
@@ -1739,14 +1670,14 @@
       <c r="C11" s="1">
         <v>125336.7</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>45385.6670148843</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -1815,6 +1746,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600" verticalDpi="600"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.700787401574803" right="0.700787401574803" top="0.751968503937008" bottom="0.751968503937008" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600" verticalDpi="600"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -1843,7 +1787,7 @@
       <c r="C1" s="1">
         <v>81847.8</v>
       </c>
-      <c r="D1" s="6">
+      <c r="D1" s="3">
         <v>44996.6670148727</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -1864,7 +1808,7 @@
       <c r="C2" s="1">
         <v>52317.9</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>45182.6670148843</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -1885,14 +1829,14 @@
       <c r="C3" s="1">
         <v>85773.6</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>45068.6670148843</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" ref="F3:F4" si="0">TRUE()</f>
         <v>1</v>
       </c>
     </row>
@@ -1906,14 +1850,14 @@
       <c r="C4" s="1">
         <v>87183</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>45349.6670148843</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F4" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
@@ -1927,7 +1871,7 @@
       <c r="C5" s="1">
         <v>30107.7</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>45054.6670148843</v>
       </c>
       <c r="E5" s="1" t="s">
@@ -1948,7 +1892,7 @@
       <c r="C6" s="1">
         <v>-1908.9</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>45167.6670148843</v>
       </c>
       <c r="E6" s="1" t="s">
@@ -1969,14 +1913,14 @@
       <c r="C7" s="1">
         <v>41974.2</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>44676.6670148843</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" ref="F7:F8" si="1">FALSE()</f>
         <v>0</v>
       </c>
     </row>
@@ -1990,14 +1934,14 @@
       <c r="C8" s="1">
         <v>128266.2</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>45743.6670148843</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F8" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2011,14 +1955,14 @@
       <c r="C9" s="1">
         <v>133728.3</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>45378.6670148843</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" ref="F9:F10" si="2">TRUE()</f>
         <v>1</v>
       </c>
     </row>
@@ -2032,14 +1976,14 @@
       <c r="C10" s="1">
         <v>125336.7</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>45385.6670148843</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -2069,7 +2013,7 @@
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="17" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="1" t="b">
@@ -2109,249 +2053,249 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="7"/>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="8"/>
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" ht="27" customHeight="1" spans="1:7">
-      <c r="A2" s="7"/>
-      <c r="B2" s="9" t="s">
+      <c r="A2" s="4"/>
+      <c r="B2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="8"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="5"/>
     </row>
     <row r="3" ht="60" spans="1:7">
-      <c r="A3" s="7"/>
-      <c r="B3" s="10" t="s">
+      <c r="A3" s="4"/>
+      <c r="B3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="7"/>
-      <c r="B4" s="11" t="s">
+      <c r="A4" s="4"/>
+      <c r="B4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="12" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="12"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="8"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="7"/>
-      <c r="B5" s="13" t="s">
+      <c r="A5" s="4"/>
+      <c r="B5" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="14" t="s">
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="8"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="5"/>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="7"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="8"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="7"/>
-      <c r="B7" s="16" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" ht="30" spans="1:7">
+      <c r="A7" s="4"/>
+      <c r="B7" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="7"/>
-      <c r="G7" s="8"/>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="7"/>
-      <c r="B8" s="17">
+      <c r="F7" s="4"/>
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" ht="28.5" spans="1:7">
+      <c r="A8" s="4"/>
+      <c r="B8" s="14">
         <v>1</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="7"/>
-      <c r="G8" s="8"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="7"/>
-      <c r="B9" s="17">
+      <c r="F8" s="4"/>
+      <c r="G8" s="5"/>
+    </row>
+    <row r="9" ht="28.5" spans="1:7">
+      <c r="A9" s="4"/>
+      <c r="B9" s="14">
         <v>1</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="16">
         <v>45301</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="5"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="7"/>
-      <c r="B10" s="17">
+      <c r="A10" s="4"/>
+      <c r="B10" s="14">
         <v>1</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="16">
         <v>45303</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="8"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="5"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="7"/>
-      <c r="B11" s="17">
+      <c r="A11" s="4"/>
+      <c r="B11" s="14">
         <v>0.5</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="16">
         <v>45306</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="5"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="7"/>
-      <c r="B12" s="17">
+      <c r="A12" s="4"/>
+      <c r="B12" s="14">
         <v>0</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="16">
         <v>45311</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="5"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="7"/>
-      <c r="B13" s="17">
+      <c r="A13" s="4"/>
+      <c r="B13" s="14">
         <v>0</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="16">
         <v>45311</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="7"/>
-      <c r="G13" s="8"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="7"/>
-      <c r="B14" s="17">
+      <c r="A14" s="4"/>
+      <c r="B14" s="14">
         <v>0</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="16">
         <v>45314</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="7"/>
-      <c r="G14" s="8"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="7"/>
-      <c r="B15" s="17">
+      <c r="A15" s="4"/>
+      <c r="B15" s="14">
         <v>0</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="16">
         <v>45316</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="7"/>
-      <c r="G15" s="8"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="5"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="7"/>
-      <c r="B16" s="17">
+      <c r="A16" s="4"/>
+      <c r="B16" s="14">
         <v>0</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="7"/>
-      <c r="G16" s="8"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="5"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="8"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2416,7 +2360,7 @@
       <c r="C2" s="1">
         <v>81847.8</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>44996.6670148727</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -2429,7 +2373,7 @@
       <c r="G2" s="1">
         <v>646</v>
       </c>
-      <c r="J2" s="6"/>
+      <c r="J2" s="3"/>
     </row>
     <row r="3" customHeight="1" spans="1:10">
       <c r="A3" s="1">
@@ -2441,7 +2385,7 @@
       <c r="C3" s="1">
         <v>52317.9</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>45182.6670148843</v>
       </c>
       <c r="E3" s="1" t="s">
@@ -2454,7 +2398,7 @@
       <c r="G3" s="1">
         <v>930</v>
       </c>
-      <c r="J3" s="6"/>
+      <c r="J3" s="3"/>
     </row>
     <row r="4" customHeight="1" spans="1:10">
       <c r="A4" s="1">
@@ -2466,20 +2410,20 @@
       <c r="C4" s="1">
         <v>85773.6</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>45068.6670148843</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" ref="F4:F5" si="0">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G4" s="1">
         <v>69</v>
       </c>
-      <c r="J4" s="6"/>
+      <c r="J4" s="3"/>
     </row>
     <row r="5" customHeight="1" spans="1:10">
       <c r="A5" s="1">
@@ -2491,20 +2435,20 @@
       <c r="C5" s="1">
         <v>87183</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>45349.6670148843</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G5" s="1">
         <v>138</v>
       </c>
-      <c r="J5" s="6"/>
+      <c r="J5" s="3"/>
     </row>
     <row r="6" customHeight="1" spans="1:10">
       <c r="A6" s="1">
@@ -2516,7 +2460,7 @@
       <c r="C6" s="1">
         <v>30107.7</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>45054.6670148843</v>
       </c>
       <c r="E6" s="1" t="s">
@@ -2529,7 +2473,7 @@
       <c r="G6" s="1">
         <v>424</v>
       </c>
-      <c r="J6" s="6"/>
+      <c r="J6" s="3"/>
     </row>
     <row r="7" customHeight="1" spans="1:10">
       <c r="A7" s="1">
@@ -2541,7 +2485,7 @@
       <c r="C7" s="1">
         <v>-1908.9</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>45167.6670148843</v>
       </c>
       <c r="E7" s="1" t="s">
@@ -2554,7 +2498,7 @@
       <c r="G7" s="1">
         <v>133</v>
       </c>
-      <c r="J7" s="6"/>
+      <c r="J7" s="3"/>
     </row>
     <row r="8" customHeight="1" spans="1:12">
       <c r="A8" s="1">
@@ -2566,27 +2510,27 @@
       <c r="C8" s="1">
         <v>41974.2</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>44676.6670148843</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" ref="F8:F9" si="1">FALSE()</f>
         <v>0</v>
       </c>
       <c r="G8" s="1">
         <v>880</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="3">
         <v>44676.6670148843</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="L8" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" ref="L8:L9" si="2">FALSE()</f>
         <v>0</v>
       </c>
     </row>
@@ -2600,27 +2544,27 @@
       <c r="C9" s="1">
         <v>128266.2</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>45743.6670148843</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G9" s="1">
         <v>954</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="3">
         <v>45743.6670148843</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="L9" s="1" t="b">
-        <f>FALSE()</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2634,27 +2578,27 @@
       <c r="C10" s="1">
         <v>133728.3</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>45378.6670148843</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F10" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" ref="F10:F11" si="3">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G10" s="1">
         <v>877</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="3">
         <v>45378.6670148843</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L10" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" ref="L10:L11" si="4">TRUE()</f>
         <v>1</v>
       </c>
     </row>
@@ -2668,27 +2612,27 @@
       <c r="C11" s="1">
         <v>125336.7</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>45385.6670148843</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G11" s="1">
         <v>339</v>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="3">
         <v>45385.6670148843</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="L11" s="1" t="b">
-        <f>TRUE()</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
     </row>
@@ -2706,68 +2650,68 @@
   <sheetFormatPr defaultColWidth="9.07619047619048" defaultRowHeight="15" customHeight="1" outlineLevelRow="5" outlineLevelCol="6"/>
   <sheetData>
     <row r="1" customHeight="1" spans="1:7">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" customHeight="1" spans="1:7">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
     </row>
     <row r="3" customHeight="1" spans="1:7">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4" t="s">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" customHeight="1" spans="1:7">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4" t="s">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="5" customHeight="1" spans="1:7">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
     </row>
     <row r="6" customHeight="1" spans="1:7">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="4" t="s">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2783,132 +2727,132 @@
   <sheetFormatPr defaultColWidth="11.5047619047619" defaultRowHeight="12.8" customHeight="1" outlineLevelRow="4" outlineLevelCol="7"/>
   <sheetData>
     <row r="1" ht="15" spans="1:8">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="1" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" ht="15" spans="1:8">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="3" ht="15" spans="1:8">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="1" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" ht="15" spans="1:8">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="1" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="5" ht="15" spans="1:8">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="1" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2940,24 +2884,24 @@
       </c>
     </row>
     <row r="2" ht="15" spans="1:3">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>2</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="3" ht="15" spans="1:9">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>5</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>6</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>7</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -2977,25 +2921,25 @@
       </c>
     </row>
     <row r="4" ht="15" spans="1:9">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>9</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>10</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>11</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>1</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <v>2</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>3</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <v>4</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -3003,16 +2947,16 @@
       </c>
     </row>
     <row r="5" ht="15" spans="5:9">
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>5</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
         <v>6</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <v>7</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="2">
         <v>8</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -3020,16 +2964,16 @@
       </c>
     </row>
     <row r="6" ht="15" spans="5:9">
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <v>9</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <v>10</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <v>11</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="2">
         <v>12</v>
       </c>
       <c r="I6" s="2" t="s">

</xml_diff>